<commit_message>
feat: substituicao do k-means por indice composto linear no ETL e refatoracao do painel
</commit_message>
<xml_diff>
--- a/Dados Tratados .xlsx
+++ b/Dados Tratados .xlsx
@@ -1,33 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Levs\mvi_ibge_prog\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD0F4A31-953D-43F3-9591-D4F87A58DC37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Página1" sheetId="1" r:id="rId5"/>
+    <sheet name="Página1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
-    <t xml:space="preserve">Estado </t>
-  </si>
-  <si>
     <t>Taxa de MVI</t>
   </si>
   <si>
     <t>Renda</t>
   </si>
   <si>
-    <t xml:space="preserve">Gini </t>
-  </si>
-  <si>
-    <t>Desmprego Médio 2024</t>
-  </si>
-  <si>
     <t>Acre</t>
   </si>
   <si>
@@ -188,28 +188,39 @@
   </si>
   <si>
     <t>1737</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Gini</t>
+  </si>
+  <si>
+    <t>Desemprego Médio 2024</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -219,11 +230,17 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -237,40 +254,40 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -278,7 +295,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -468,45 +485,48 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="5" max="5" width="19.63"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" s="3">
+        <v>20.326334185373899</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3">
-        <v>20.3263341853739</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>6</v>
       </c>
       <c r="D2" s="5">
         <v>0.502</v>
@@ -515,117 +535,117 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B3" s="3">
-        <v>35.43363816820823</v>
+        <v>35.433638168208233</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D3" s="5">
-        <v>0.516</v>
+        <v>0.51600000000000001</v>
       </c>
       <c r="E3" s="5">
         <v>8.5</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B4" s="3">
         <v>45.090099235585804</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D4" s="5">
-        <v>0.509</v>
+        <v>0.50900000000000001</v>
       </c>
       <c r="E4" s="5">
-        <v>9.2</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B5" s="3">
         <v>27.398802534517703</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D5" s="5">
-        <v>0.474</v>
+        <v>0.47399999999999998</v>
       </c>
       <c r="E5" s="5">
-        <v>8.575</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>8.5749999999999993</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B6" s="3">
         <v>40.645060544373116</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D6" s="5">
-        <v>0.477</v>
+        <v>0.47699999999999998</v>
       </c>
       <c r="E6" s="5">
-        <v>11.175</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>11.175000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B7" s="3">
         <v>37.547424335496146</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D7" s="5">
-        <v>0.487</v>
+        <v>0.48699999999999999</v>
       </c>
       <c r="E7" s="5">
         <v>7.35</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3">
+        <v>8.9177415450758311</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="5">
+        <v>0.54700000000000004</v>
+      </c>
+      <c r="E8" s="5">
+        <v>9.3249999999999993</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="3">
+        <v>23.890033687385259</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="B8" s="3">
-        <v>8.917741545075831</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="5">
-        <v>0.547</v>
-      </c>
-      <c r="E8" s="5">
-        <v>9.325</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="3">
-        <v>23.89003368738526</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>20</v>
       </c>
       <c r="D9" s="5">
         <v>0.48</v>
@@ -634,49 +654,49 @@
         <v>4.625</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B10" s="3">
         <v>18.760671917750166</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D10" s="5">
-        <v>0.462</v>
+        <v>0.46200000000000002</v>
       </c>
       <c r="E10" s="5">
         <v>5.35</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="3">
+        <v>30.366740075538871</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="5">
+        <v>0.48699999999999999</v>
+      </c>
+      <c r="E11" s="5">
+        <v>7.5749999999999993</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3">
+        <v>29.767498114768561</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="B11" s="3">
-        <v>30.36674007553887</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="5">
-        <v>0.487</v>
-      </c>
-      <c r="E11" s="5">
-        <v>7.574999999999999</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="3">
-        <v>29.76749811476856</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="D12" s="5">
         <v>0.442</v>
@@ -685,49 +705,49 @@
         <v>2.9749999999999996</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B13" s="3">
         <v>18.746370905908034</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D13" s="5">
-        <v>0.454</v>
+        <v>0.45400000000000001</v>
       </c>
       <c r="E13" s="5">
         <v>3.9750000000000005</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B14" s="3">
         <v>15.073144379384386</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D14" s="5">
-        <v>0.447</v>
+        <v>0.44700000000000001</v>
       </c>
       <c r="E14" s="5">
         <v>5.2250000000000005</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B15" s="3">
         <v>29.546509553102116</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D15" s="5">
         <v>0.49</v>
@@ -736,49 +756,49 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B16" s="3">
         <v>25.57273271186768</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D16" s="5">
         <v>0.496</v>
       </c>
       <c r="E16" s="5">
-        <v>8.725000000000001</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>8.7250000000000014</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B17" s="3">
         <v>18.351471267896386</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D17" s="5">
-        <v>0.473</v>
+        <v>0.47299999999999998</v>
       </c>
       <c r="E17" s="5">
-        <v>4.1</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B18" s="3">
         <v>36.19865292368857</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D18" s="5">
         <v>0.53</v>
@@ -787,83 +807,83 @@
         <v>11.225000000000001</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B19" s="3">
         <v>20.292412178291208</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D19" s="5">
-        <v>0.493</v>
+        <v>0.49299999999999999</v>
       </c>
       <c r="E19" s="5">
-        <v>8.275</v>
-      </c>
-    </row>
-    <row r="20">
+        <v>8.2750000000000004</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B20" s="3">
         <v>22.120040681362294</v>
       </c>
       <c r="C20" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="5">
+        <v>0.52200000000000002</v>
+      </c>
+      <c r="E20" s="5">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="3">
+        <v>24.172456110161399</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" s="5">
+        <v>0.52200000000000002</v>
+      </c>
+      <c r="E21" s="5">
+        <v>9.1499999999999986</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D20" s="5">
-        <v>0.522</v>
-      </c>
-      <c r="E20" s="5">
-        <v>9.2</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B21" s="3">
-        <v>24.1724561101614</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" s="5">
-        <v>0.522</v>
-      </c>
-      <c r="E21" s="5">
-        <v>9.149999999999999</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="s">
-        <v>45</v>
       </c>
       <c r="B22" s="3">
         <v>15.022375503287424</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D22" s="5">
-        <v>0.458</v>
+        <v>0.45800000000000002</v>
       </c>
       <c r="E22" s="5">
-        <v>5.324999999999999</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>5.3249999999999993</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B23" s="3">
         <v>26.05617711786612</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D23" s="5">
         <v>0.442</v>
@@ -872,15 +892,15 @@
         <v>2.95</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B24" s="3">
         <v>18.554868699889646</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D24" s="5">
         <v>0.53</v>
@@ -889,15 +909,15 @@
         <v>6.9</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B25" s="3">
-        <v>8.50040348995544</v>
+        <v>8.5004034899554402</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D25" s="5">
         <v>0.43</v>
@@ -906,58 +926,58 @@
         <v>3.1499999999999995</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B26" s="3">
-        <v>8.159102454356336</v>
+        <v>8.1591024543563364</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D26" s="5">
-        <v>0.489</v>
+        <v>0.48899999999999999</v>
       </c>
       <c r="E26" s="5">
-        <v>6.449999999999999</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>6.4499999999999993</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B27" s="3">
         <v>22.784044359923303</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D27" s="5">
         <v>0.498</v>
       </c>
       <c r="E27" s="5">
-        <v>9.0</v>
-      </c>
-    </row>
-    <row r="28">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B28" s="3">
         <v>19.780111098290668</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D28" s="5">
-        <v>0.477</v>
+        <v>0.47699999999999998</v>
       </c>
       <c r="E28" s="5">
         <v>5.1499999999999995</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>